<commit_message>
Version estable con instalador
</commit_message>
<xml_diff>
--- a/Formato SV.xlsx
+++ b/Formato SV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avjimenez\Desktop\Magnus_RPA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DFB191-B3F8-4914-A6A1-61BC5F01E873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43B2E92-5788-4FA9-BFF7-9E8CC9F9DEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C0B68480-AD38-469B-85F4-40DE2CF20192}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>sociedad</t>
   </si>
@@ -86,10 +86,19 @@
     <t>PX 22.09.2026</t>
   </si>
   <si>
-    <t>24.09.2026</t>
-  </si>
-  <si>
     <t>usuario_sap</t>
+  </si>
+  <si>
+    <t>101753467</t>
+  </si>
+  <si>
+    <t>101999932</t>
+  </si>
+  <si>
+    <t>01.10.2026</t>
+  </si>
+  <si>
+    <t>01.10.2027</t>
   </si>
 </sst>
 </file>
@@ -99,7 +108,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +128,20 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -170,7 +193,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -187,6 +210,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -522,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF75257A-32E8-4FA1-8177-5B7B1205B374}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -554,7 +579,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -573,14 +598,14 @@
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="5">
-        <v>101848405</v>
+      <c r="B2" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>150</v>
+        <v>266.05</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -599,14 +624,14 @@
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3">
-        <v>101912486</v>
+      <c r="B3" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3">
-        <v>350</v>
+        <v>90</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -621,7 +646,22 @@
         <v>2151</v>
       </c>
     </row>
+    <row r="4" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>